<commit_message>
Rebuild Mobility document summary without AI-based MLB
Keep only the eRAN21.1 Idle / Connected / Intra-RAT MLB feature
summary in the operator Excel format. Remove the Daily KPI agent
sheet and all AI-based load-balance workflow content.

Co-authored-by: Mohammad Selim <miles4482@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/4G_LTE_Mobility_Management/Mobility_Management_eRAN21.1_Workbook.xlsx
+++ b/docs/4G_LTE_Mobility_Management/Mobility_Management_eRAN21.1_Workbook.xlsx
@@ -11,7 +11,6 @@
     <sheet name="Idle Mode Management" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Connected Mode" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Intra-RAT MLB" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Daily KPI" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -112,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -130,12 +129,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -211,203 +204,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>High / Low / Close (example — replace with live BH)</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Daily KPI'!C36</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="5B9BD5"/>
-            </a:solidFill>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Daily KPI'!$A$37:$A$43</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Daily KPI'!$C$37:$C$43</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>'Daily KPI'!D36</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="A9D08E"/>
-            </a:solidFill>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Daily KPI'!$A$37:$A$43</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Daily KPI'!$D$37:$D$43</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="2"/>
-          <order val="2"/>
-          <tx>
-            <strRef>
-              <f>'Daily KPI'!E36</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="F4B183"/>
-            </a:solidFill>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Daily KPI'!$A$37:$A$43</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Daily KPI'!$E$37:$E$43</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Date</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Mbps</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>54</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="6480000" cy="2880000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -700,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -788,22 +584,22 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Intra-LTE mobility + MLB</t>
+          <t>Document summary of Mobility Management</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>DL user-throughput gap among capacity layers</t>
+          <t>Idle Mode + Connected Mode + Intra-RAT MLB</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Target 1-2 Mbps (now &gt;10 Mbps worst cells)</t>
+          <t>Huawei eRAN21.1 feature books</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>Gap &gt; 2 Mbps is an investigation trigger, not automatic proof that A1-A4 or MLB must change.</t>
+          <t>Parameter and feature summary from the three eRAN21.1 Mobility Management documents. SN-1 to SN-11 on each feature sheet.</t>
         </is>
       </c>
     </row>
@@ -921,7 +717,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Idle Mode / Connected Mode / Intra-RAT MLB / Daily KPI</t>
+          <t>Idle Mode Management / Connected Mode / Intra-RAT MLB</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -990,12 +786,12 @@
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>Calibrate before live CR</t>
+          <t>Calibrate before live change</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Rollback if drop, VoLTE, re-est, HO success or L900 indoor KPI degrades. Do not daily overwrite 7-day learned MLB thresholds.</t>
+          <t>Rollback if drop, VoLTE, re-est, HO success or L900 indoor KPI degrades. Huawei learned MLB thresholds collect 7 days and refresh every 7 days — do not overwrite them every day.</t>
         </is>
       </c>
     </row>
@@ -1215,7 +1011,7 @@
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>Typical Open value on Daily KPI sheet.</t>
+          <t>Typical fallback below L2600 when high-band load is high.</t>
         </is>
       </c>
     </row>
@@ -1500,38 +1296,6 @@
       <c r="F31" s="7" t="inlineStr">
         <is>
           <t>Chart / doc ref is in the last column (Notes).</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="28" customHeight="1">
-      <c r="A32" s="7" t="inlineStr">
-        <is>
-          <t>Daily KPI</t>
-        </is>
-      </c>
-      <c r="B32" s="7" t="inlineStr">
-        <is>
-          <t>LTE FDD</t>
-        </is>
-      </c>
-      <c r="C32" s="7" t="inlineStr">
-        <is>
-          <t>Date / Open / High / Low / Close</t>
-        </is>
-      </c>
-      <c r="D32" s="7" t="inlineStr">
-        <is>
-          <t>Open=L1800 TP, High=max layer, Low=min layer, Close=gap</t>
-        </is>
-      </c>
-      <c r="E32" s="7" t="inlineStr">
-        <is>
-          <t>Investigate if Close&gt;2</t>
-        </is>
-      </c>
-      <c r="F32" s="7" t="inlineStr">
-        <is>
-          <t>L900 is not included in High/Low.</t>
         </is>
       </c>
     </row>
@@ -7394,7 +7158,7 @@
     <row r="48" ht="26" customHeight="1">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>Smart learned thd</t>
+          <t>Huawei learned neighbor thd</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
@@ -7409,7 +7173,7 @@
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>Freeze AI CRs in relearn week</t>
+          <t>Allow 7-day relearn after those events</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
@@ -7417,7 +7181,11 @@
           <t>Stale or reset [MLB] pp.29-31</t>
         </is>
       </c>
-      <c r="F48" s="7" t="inlineStr"/>
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>Huawei native NCellTrigThldSmartOptAlgoSw. Collects 7 days, recalculates every 7 days.</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="26" customHeight="1">
       <c r="A49" s="7" t="inlineStr">
@@ -7634,7 +7402,7 @@
     <row r="58" ht="22" customHeight="1">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>Smart n-cell thd</t>
+          <t>Huawei learned n-cell thd</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
@@ -7649,15 +7417,19 @@
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>SON MLB option + MAE counters</t>
+          <t>Huawei option + MAE 15-min counters</t>
         </is>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>AI monitors, no daily MOD</t>
-        </is>
-      </c>
-      <c r="F58" s="7" t="inlineStr"/>
+          <t>Optional; 7-day learn / 7-day refresh</t>
+        </is>
+      </c>
+      <c r="F58" s="7" t="inlineStr">
+        <is>
+          <t>Do not overwrite learned pair thresholds every day.</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="12" customHeight="1">
       <c r="A59" s="3" t="inlineStr"/>
@@ -7995,7 +7767,7 @@
       </c>
       <c r="F71" s="7" t="inlineStr">
         <is>
-          <t>MAIN daily CR. Do not copy 20 MHz thd to L2100.</t>
+          <t>Do not copy a 20 MHz threshold onto L2100.</t>
         </is>
       </c>
     </row>
@@ -8168,7 +7940,7 @@
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>smart</t>
+          <t>CELLMLB / related</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
@@ -8178,12 +7950,12 @@
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>Monitor only daily</t>
+          <t>Optional Huawei function</t>
         </is>
       </c>
       <c r="F77" s="7" t="inlineStr">
         <is>
-          <t>7-day learn. No daily overwrite.</t>
+          <t>7-day data collection, then refresh every 7 days.</t>
         </is>
       </c>
     </row>
@@ -8499,7 +8271,7 @@
       </c>
       <c r="F89" s="7" t="inlineStr">
         <is>
-          <t>MAIN guarded CR. Do not copy 20 MHz thd to L2100.</t>
+          <t>Do not copy a 20 MHz threshold onto L2100.</t>
         </is>
       </c>
     </row>
@@ -8694,1205 +8466,4 @@
     <firstFooter/>
   </headerFooter>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="00005596"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:F54"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="54" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Daily KPI - Date / Open / High / Low / Close Detailed Notes</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="12" customHeight="1">
-      <c r="A2" s="3" t="inlineStr"/>
-      <c r="B2" s="3" t="inlineStr"/>
-      <c r="C2" s="3" t="inlineStr"/>
-      <c r="D2" s="3" t="inlineStr"/>
-      <c r="E2" s="3" t="inlineStr"/>
-      <c r="F2" s="3" t="inlineStr"/>
-    </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Section 1: Feature Introduction</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="n"/>
-      <c r="C3" s="5" t="n"/>
-      <c r="D3" s="5" t="n"/>
-      <c r="E3" s="5" t="n"/>
-      <c r="F3" s="5" t="n"/>
-    </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>Topic</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>RAT</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>Feature Part</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>Parameter ID / Check Item</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>Current Value / Status</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>Notes / Rationale</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>LTE FDD</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>Busy-hour date</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>KPI date</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>Fill daily</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>White-on-blue title only. Table uses the attached light format.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>LTE FDD</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>Anchor layer TP</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>L1800 DL user throughput Mbps</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>Capacity layer</t>
-        </is>
-      </c>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>Change to L2100 if L1800 is missing on that sector.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>LTE FDD</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>Best capacity layer</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>Max DL user TP among L1800/L2100/L2600 C1-C4</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>Mbps</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>Do not include L900.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>LTE FDD</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Worst capacity layer</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>Min DL user TP among capacity layers</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>Mbps</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>Worst cell/layer for the gap.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>Close</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>LTE FDD</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>Throughput gap</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>High minus Low</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>Investigate if Close &gt; 2 Mbps</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>CR only after RCA pass. Not automatic MLB change.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="12" customHeight="1">
-      <c r="A10" s="3" t="inlineStr"/>
-      <c r="B10" s="3" t="inlineStr"/>
-      <c r="C10" s="3" t="inlineStr"/>
-      <c r="D10" s="3" t="inlineStr"/>
-      <c r="E10" s="3" t="inlineStr"/>
-      <c r="F10" s="3" t="inlineStr"/>
-    </row>
-    <row r="11" ht="12" customHeight="1">
-      <c r="A11" s="3" t="inlineStr"/>
-      <c r="B11" s="3" t="inlineStr"/>
-      <c r="C11" s="3" t="inlineStr"/>
-      <c r="D11" s="3" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr"/>
-      <c r="F11" s="3" t="inlineStr"/>
-    </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Section 2: Triggering Conditions  (RCA when Close &gt; 2 Mbps)</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5" t="n"/>
-    </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>Feature Part</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>RAT</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>MO Name / Check Item</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>When Power Saving Starts</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>Parameter Detail</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>User Experience Consideration</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="28" customHeight="1">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>Class 1 Load / PCell</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>LTE FDD</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>Active UE + PRB + spare target C</t>
-        </is>
-      </c>
-      <c r="D14" s="7" t="inlineStr">
-        <is>
-          <t>Low TP + high PRB + high users; target spare + good overlap</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="inlineStr">
-        <is>
-          <t>YES — Feature 3</t>
-        </is>
-      </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t>Active-UE MLB / LOADPRIORITY / modest thd. Column name from template = when the check starts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="28" customHeight="1">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>Class 2 Heavy-user PRB</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>LTE FDD</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>Few UEs, very high PRB, non-CA</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>PRB supplement only</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>YES only as supplement</t>
-        </is>
-      </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>Never sole algorithm if CA high.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>Class 3 CA / SCell</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>LTE FDD</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="inlineStr">
-        <is>
-          <t>PCell vs SCell / active CC</t>
-        </is>
-      </c>
-      <c r="D16" s="7" t="inlineStr">
-        <is>
-          <t>PCell looks bad but SCell healthy, or SCell never on</t>
-        </is>
-      </c>
-      <c r="E16" s="7" t="inlineStr">
-        <is>
-          <t>NO first</t>
-        </is>
-      </c>
-      <c r="F16" s="7" t="inlineStr">
-        <is>
-          <t>CA combo / activation / scheduler.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="28" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>Class 4 RF / interference</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>LTE FDD</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="inlineStr">
-        <is>
-          <t>CQI / SINR / RSRP</t>
-        </is>
-      </c>
-      <c r="D17" s="7" t="inlineStr">
-        <is>
-          <t>Low TP + low CQI, PRB not high</t>
-        </is>
-      </c>
-      <c r="E17" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F17" s="7" t="inlineStr">
-        <is>
-          <t>RF / PCI / overshoot / external.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>Class 5 UE capability</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>LTE FDD</t>
-        </is>
-      </c>
-      <c r="C18" s="7" t="inlineStr">
-        <is>
-          <t>Band support</t>
-        </is>
-      </c>
-      <c r="D18" s="7" t="inlineStr">
-        <is>
-          <t>L2600 empty because UEs have no band</t>
-        </is>
-      </c>
-      <c r="E18" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F18" s="7" t="inlineStr">
-        <is>
-          <t>Device mix.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="28" customHeight="1">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>Class 6 Mobility / meas</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>LTE FDD</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="inlineStr">
-        <is>
-          <t>Prep/Exec/MeasSucc</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>High Prep, low Exec</t>
-        </is>
-      </c>
-      <c r="E19" s="7" t="inlineStr">
-        <is>
-          <t>NO until flags/NRT/A4 fixed</t>
-        </is>
-      </c>
-      <c r="F19" s="7" t="inlineStr">
-        <is>
-          <t>Connected Mode audit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="28" customHeight="1">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>Class 7 HW / transport</t>
-        </is>
-      </c>
-      <c r="B20" s="7" t="inlineStr">
-        <is>
-          <t>LTE FDD</t>
-        </is>
-      </c>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>Alarms / HighLoad transport</t>
-        </is>
-      </c>
-      <c r="D20" s="7" t="inlineStr">
-        <is>
-          <t>Low TP, resources look free</t>
-        </is>
-      </c>
-      <c r="E20" s="7" t="inlineStr">
-        <is>
-          <t>NO — illegal target</t>
-        </is>
-      </c>
-      <c r="F20" s="7" t="inlineStr">
-        <is>
-          <t>Clear alarm first.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="28" customHeight="1">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>Class 8 L900 indoor</t>
-        </is>
-      </c>
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>LTE FDD</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>High-band MR poor</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>Users survive only on L900</t>
-        </is>
-      </c>
-      <c r="E21" s="7" t="inlineStr">
-        <is>
-          <t>NO forced offload</t>
-        </is>
-      </c>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>RF / indoor. A1-escape only if overlap is strong.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="12" customHeight="1">
-      <c r="A22" s="3" t="inlineStr"/>
-      <c r="B22" s="3" t="inlineStr"/>
-      <c r="C22" s="3" t="inlineStr"/>
-      <c r="D22" s="3" t="inlineStr"/>
-      <c r="E22" s="3" t="inlineStr"/>
-      <c r="F22" s="3" t="inlineStr"/>
-    </row>
-    <row r="23" ht="12" customHeight="1">
-      <c r="A23" s="3" t="inlineStr"/>
-      <c r="B23" s="3" t="inlineStr"/>
-      <c r="C23" s="3" t="inlineStr"/>
-      <c r="D23" s="3" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="3" t="inlineStr"/>
-    </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>Section 3: eNodeB Actions  (approval rule and least-invasive CR)</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="n"/>
-      <c r="C24" s="5" t="n"/>
-      <c r="D24" s="5" t="n"/>
-      <c r="E24" s="5" t="n"/>
-      <c r="F24" s="5" t="n"/>
-    </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>Action Area</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>RAT</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="inlineStr">
-        <is>
-          <t>Feature Part</t>
-        </is>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>eNodeB Action</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="inlineStr">
-        <is>
-          <t>Parameter / Condition</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>Operational Meaning</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="7" t="inlineStr">
-        <is>
-          <t>Approval rule</t>
-        </is>
-      </c>
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t>LTE FDD</t>
-        </is>
-      </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>Daily agent</t>
-        </is>
-      </c>
-      <c r="D26" s="7" t="inlineStr">
-        <is>
-          <t>CR only if Close&gt;2 AND sustained AND source load high AND target spare C AND target RF OK AND HO healthy AND no alarm AND drop/VoLTE/re-est/L900 OK</t>
-        </is>
-      </c>
-      <c r="E26" s="7" t="inlineStr">
-        <is>
-          <t>All must be true</t>
-        </is>
-      </c>
-      <c r="F26" s="7" t="inlineStr">
-        <is>
-          <t>Else RCA only. One parameter family per cluster.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>Order 1</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>LTE FDD</t>
-        </is>
-      </c>
-      <c r="C27" s="7" t="inlineStr">
-        <is>
-          <t>Eligibility</t>
-        </is>
-      </c>
-      <c r="D27" s="7" t="inlineStr">
-        <is>
-          <t>Fix NRT / meas flag / L900 wrongly set as MLB target</t>
-        </is>
-      </c>
-      <c r="E27" s="7" t="inlineStr">
-        <is>
-          <t>F2+F3 MML step 1-2</t>
-        </is>
-      </c>
-      <c r="F27" s="7" t="inlineStr">
-        <is>
-          <t>Most silent failures.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="7" t="inlineStr">
-        <is>
-          <t>Order 2</t>
-        </is>
-      </c>
-      <c r="B28" s="7" t="inlineStr">
-        <is>
-          <t>LTE FDD</t>
-        </is>
-      </c>
-      <c r="C28" s="7" t="inlineStr">
-        <is>
-          <t>Load model</t>
-        </is>
-      </c>
-      <c r="D28" s="7" t="inlineStr">
-        <is>
-          <t>Turn ON ActiveUe + SpectralEff</t>
-        </is>
-      </c>
-      <c r="E28" s="7" t="inlineStr">
-        <is>
-          <t>F3 Section 3</t>
-        </is>
-      </c>
-      <c r="F28" s="7" t="inlineStr">
-        <is>
-          <t>Required on 15 vs 20 MHz.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="7" t="inlineStr">
-        <is>
-          <t>Order 3</t>
-        </is>
-      </c>
-      <c r="B29" s="7" t="inlineStr">
-        <is>
-          <t>LTE FDD</t>
-        </is>
-      </c>
-      <c r="C29" s="7" t="inlineStr">
-        <is>
-          <t>Trigger / volume</t>
-        </is>
-      </c>
-      <c r="D29" s="7" t="inlineStr">
-        <is>
-          <t>Modest InterFreqMlbUeNumThd / offset / MlbMaxUeNum</t>
-        </is>
-      </c>
-      <c r="E29" s="7" t="inlineStr">
-        <is>
-          <t>After load model ON</t>
-        </is>
-      </c>
-      <c r="F29" s="7" t="inlineStr">
-        <is>
-          <t>MAIN daily CR.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="7" t="inlineStr">
-        <is>
-          <t>Order 4</t>
-        </is>
-      </c>
-      <c r="B30" s="7" t="inlineStr">
-        <is>
-          <t>LTE FDD</t>
-        </is>
-      </c>
-      <c r="C30" s="7" t="inlineStr">
-        <is>
-          <t>Four L2600</t>
-        </is>
-      </c>
-      <c r="D30" s="7" t="inlineStr">
-        <is>
-          <t>LOADPRIORITY; equal idle priority</t>
-        </is>
-      </c>
-      <c r="E30" s="7" t="inlineStr">
-        <is>
-          <t>Load exchange OK</t>
-        </is>
-      </c>
-      <c r="F30" s="7" t="inlineStr">
-        <is>
-          <t>Not static C1&gt;C2&gt;C3&gt;C4.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="7" t="inlineStr">
-        <is>
-          <t>Order 5-7</t>
-        </is>
-      </c>
-      <c r="B31" s="7" t="inlineStr">
-        <is>
-          <t>LTE FDD</t>
-        </is>
-      </c>
-      <c r="C31" s="7" t="inlineStr">
-        <is>
-          <t>CA / idle bounce / L900 sticky</t>
-        </is>
-      </c>
-      <c r="D31" s="7" t="inlineStr">
-        <is>
-          <t>CaUserLoadTransfer after audit; idle T320 hold; A1/FreqPri escape</t>
-        </is>
-      </c>
-      <c r="E31" s="7" t="inlineStr">
-        <is>
-          <t>Never weaken L900 floors</t>
-        </is>
-      </c>
-      <c r="F31" s="7" t="inlineStr">
-        <is>
-          <t>Escape only where high-band MR is good.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="7" t="inlineStr">
-        <is>
-          <t>Rollback</t>
-        </is>
-      </c>
-      <c r="B32" s="7" t="inlineStr">
-        <is>
-          <t>LTE FDD</t>
-        </is>
-      </c>
-      <c r="C32" s="7" t="inlineStr">
-        <is>
-          <t>Guardrail</t>
-        </is>
-      </c>
-      <c r="D32" s="7" t="inlineStr">
-        <is>
-          <t>Rollback if L900/VoLTE/drop/HO/re-est worsen or congestion only moves</t>
-        </is>
-      </c>
-      <c r="E32" s="7" t="inlineStr">
-        <is>
-          <t>Do not daily MOD learned SON thds</t>
-        </is>
-      </c>
-      <c r="F32" s="7" t="inlineStr">
-        <is>
-          <t>Evaluate at sector-cluster level.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="12" customHeight="1">
-      <c r="A33" s="3" t="inlineStr"/>
-      <c r="B33" s="3" t="inlineStr"/>
-      <c r="C33" s="3" t="inlineStr"/>
-      <c r="D33" s="3" t="inlineStr"/>
-      <c r="E33" s="3" t="inlineStr"/>
-      <c r="F33" s="3" t="inlineStr"/>
-    </row>
-    <row r="34" ht="12" customHeight="1">
-      <c r="A34" s="3" t="inlineStr"/>
-      <c r="B34" s="3" t="inlineStr"/>
-      <c r="C34" s="3" t="inlineStr"/>
-      <c r="D34" s="3" t="inlineStr"/>
-      <c r="E34" s="3" t="inlineStr"/>
-      <c r="F34" s="3" t="inlineStr"/>
-    </row>
-    <row r="35" ht="22" customHeight="1">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>Section 4: Daily tracker  (fill Open / High / Low; Close = High − Low)</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="n"/>
-      <c r="C35" s="5" t="n"/>
-      <c r="D35" s="5" t="n"/>
-      <c r="E35" s="5" t="n"/>
-      <c r="F35" s="5" t="n"/>
-    </row>
-    <row r="36" ht="22" customHeight="1">
-      <c r="A36" s="6" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B36" s="6" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C36" s="6" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="D36" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="E36" s="6" t="inlineStr">
-        <is>
-          <t>Close</t>
-        </is>
-      </c>
-      <c r="F36" s="6" t="inlineStr">
-        <is>
-          <t>Notes / Rationale</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="8" t="inlineStr">
-        <is>
-          <t>Day-1</t>
-        </is>
-      </c>
-      <c r="B37" s="8" t="n">
-        <v>18</v>
-      </c>
-      <c r="C37" s="8" t="n">
-        <v>22</v>
-      </c>
-      <c r="D37" s="8" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="E37" s="8">
-        <f>C37-D37</f>
-        <v/>
-      </c>
-      <c r="F37" s="7" t="inlineStr">
-        <is>
-          <t>Example only — replace with live BH. Worst layer in Notes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="8" t="inlineStr">
-        <is>
-          <t>Day-2</t>
-        </is>
-      </c>
-      <c r="B38" s="8" t="n">
-        <v>17.5</v>
-      </c>
-      <c r="C38" s="8" t="n">
-        <v>21</v>
-      </c>
-      <c r="D38" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="E38" s="8">
-        <f>C38-D38</f>
-        <v/>
-      </c>
-      <c r="F38" s="7" t="inlineStr"/>
-    </row>
-    <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="8" t="inlineStr">
-        <is>
-          <t>Day-3</t>
-        </is>
-      </c>
-      <c r="B39" s="8" t="n">
-        <v>19</v>
-      </c>
-      <c r="C39" s="8" t="n">
-        <v>20.5</v>
-      </c>
-      <c r="D39" s="8" t="n">
-        <v>11.2</v>
-      </c>
-      <c r="E39" s="8">
-        <f>C39-D39</f>
-        <v/>
-      </c>
-      <c r="F39" s="7" t="inlineStr"/>
-    </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="8" t="inlineStr">
-        <is>
-          <t>Day-4</t>
-        </is>
-      </c>
-      <c r="B40" s="8" t="n">
-        <v>18.2</v>
-      </c>
-      <c r="C40" s="8" t="n">
-        <v>19.8</v>
-      </c>
-      <c r="D40" s="8" t="n">
-        <v>16</v>
-      </c>
-      <c r="E40" s="8">
-        <f>C40-D40</f>
-        <v/>
-      </c>
-      <c r="F40" s="7" t="inlineStr">
-        <is>
-          <t>Gap falling after first guarded CR.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="20" customHeight="1">
-      <c r="A41" s="8" t="inlineStr">
-        <is>
-          <t>Day-5</t>
-        </is>
-      </c>
-      <c r="B41" s="8" t="n">
-        <v>18.5</v>
-      </c>
-      <c r="C41" s="8" t="n">
-        <v>19.4</v>
-      </c>
-      <c r="D41" s="8" t="n">
-        <v>17.6</v>
-      </c>
-      <c r="E41" s="8">
-        <f>C41-D41</f>
-        <v/>
-      </c>
-      <c r="F41" s="7" t="inlineStr"/>
-    </row>
-    <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="8" t="inlineStr">
-        <is>
-          <t>Day-6</t>
-        </is>
-      </c>
-      <c r="B42" s="8" t="n">
-        <v>18.8</v>
-      </c>
-      <c r="C42" s="8" t="n">
-        <v>19.2</v>
-      </c>
-      <c r="D42" s="8" t="n">
-        <v>17.9</v>
-      </c>
-      <c r="E42" s="8">
-        <f>C42-D42</f>
-        <v/>
-      </c>
-      <c r="F42" s="7" t="inlineStr"/>
-    </row>
-    <row r="43" ht="20" customHeight="1">
-      <c r="A43" s="8" t="inlineStr">
-        <is>
-          <t>Day-7</t>
-        </is>
-      </c>
-      <c r="B43" s="8" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="C43" s="8" t="n">
-        <v>19</v>
-      </c>
-      <c r="D43" s="8" t="n">
-        <v>17.8</v>
-      </c>
-      <c r="E43" s="8">
-        <f>C43-D43</f>
-        <v/>
-      </c>
-      <c r="F43" s="7" t="inlineStr">
-        <is>
-          <t>Close near 1-2 Mbps target.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="9" t="inlineStr"/>
-      <c r="B44" s="9" t="inlineStr"/>
-      <c r="C44" s="9" t="inlineStr"/>
-      <c r="D44" s="9" t="inlineStr"/>
-      <c r="E44" s="8">
-        <f>IF(OR(C44="",D44=""),"",C44-D44)</f>
-        <v/>
-      </c>
-      <c r="F44" s="9" t="inlineStr"/>
-    </row>
-    <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="9" t="inlineStr"/>
-      <c r="B45" s="9" t="inlineStr"/>
-      <c r="C45" s="9" t="inlineStr"/>
-      <c r="D45" s="9" t="inlineStr"/>
-      <c r="E45" s="8">
-        <f>IF(OR(C45="",D45=""),"",C45-D45)</f>
-        <v/>
-      </c>
-      <c r="F45" s="9" t="inlineStr"/>
-    </row>
-    <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="9" t="inlineStr"/>
-      <c r="B46" s="9" t="inlineStr"/>
-      <c r="C46" s="9" t="inlineStr"/>
-      <c r="D46" s="9" t="inlineStr"/>
-      <c r="E46" s="8">
-        <f>IF(OR(C46="",D46=""),"",C46-D46)</f>
-        <v/>
-      </c>
-      <c r="F46" s="9" t="inlineStr"/>
-    </row>
-    <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="9" t="inlineStr"/>
-      <c r="B47" s="9" t="inlineStr"/>
-      <c r="C47" s="9" t="inlineStr"/>
-      <c r="D47" s="9" t="inlineStr"/>
-      <c r="E47" s="8">
-        <f>IF(OR(C47="",D47=""),"",C47-D47)</f>
-        <v/>
-      </c>
-      <c r="F47" s="9" t="inlineStr"/>
-    </row>
-    <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="9" t="inlineStr"/>
-      <c r="B48" s="9" t="inlineStr"/>
-      <c r="C48" s="9" t="inlineStr"/>
-      <c r="D48" s="9" t="inlineStr"/>
-      <c r="E48" s="8">
-        <f>IF(OR(C48="",D48=""),"",C48-D48)</f>
-        <v/>
-      </c>
-      <c r="F48" s="9" t="inlineStr"/>
-    </row>
-    <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="9" t="inlineStr"/>
-      <c r="B49" s="9" t="inlineStr"/>
-      <c r="C49" s="9" t="inlineStr"/>
-      <c r="D49" s="9" t="inlineStr"/>
-      <c r="E49" s="8">
-        <f>IF(OR(C49="",D49=""),"",C49-D49)</f>
-        <v/>
-      </c>
-      <c r="F49" s="9" t="inlineStr"/>
-    </row>
-    <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="9" t="inlineStr"/>
-      <c r="B50" s="9" t="inlineStr"/>
-      <c r="C50" s="9" t="inlineStr"/>
-      <c r="D50" s="9" t="inlineStr"/>
-      <c r="E50" s="8">
-        <f>IF(OR(C50="",D50=""),"",C50-D50)</f>
-        <v/>
-      </c>
-      <c r="F50" s="9" t="inlineStr"/>
-    </row>
-    <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="9" t="inlineStr"/>
-      <c r="B51" s="9" t="inlineStr"/>
-      <c r="C51" s="9" t="inlineStr"/>
-      <c r="D51" s="9" t="inlineStr"/>
-      <c r="E51" s="8">
-        <f>IF(OR(C51="",D51=""),"",C51-D51)</f>
-        <v/>
-      </c>
-      <c r="F51" s="9" t="inlineStr"/>
-    </row>
-    <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="9" t="inlineStr"/>
-      <c r="B52" s="9" t="inlineStr"/>
-      <c r="C52" s="9" t="inlineStr"/>
-      <c r="D52" s="9" t="inlineStr"/>
-      <c r="E52" s="8">
-        <f>IF(OR(C52="",D52=""),"",C52-D52)</f>
-        <v/>
-      </c>
-      <c r="F52" s="9" t="inlineStr"/>
-    </row>
-    <row r="53" ht="18" customHeight="1">
-      <c r="A53" s="9" t="inlineStr"/>
-      <c r="B53" s="9" t="inlineStr"/>
-      <c r="C53" s="9" t="inlineStr"/>
-      <c r="D53" s="9" t="inlineStr"/>
-      <c r="E53" s="8">
-        <f>IF(OR(C53="",D53=""),"",C53-D53)</f>
-        <v/>
-      </c>
-      <c r="F53" s="9" t="inlineStr"/>
-    </row>
-    <row r="54" ht="12" customHeight="1">
-      <c r="A54" s="3" t="inlineStr"/>
-      <c r="B54" s="3" t="inlineStr"/>
-      <c r="C54" s="3" t="inlineStr"/>
-      <c r="D54" s="3" t="inlineStr"/>
-      <c r="E54" s="3" t="inlineStr"/>
-      <c r="F54" s="3" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A24:F24"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A35:F35"/>
-    <mergeCell ref="A3:F3"/>
-  </mergeCells>
-  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
-  <headerFooter>
-    <oddHeader>&amp;LMobility Management</oddHeader>
-    <oddFooter>&amp;LDaily KPI&amp;RHuawei eRAN21.1  |  Page &amp;P of &amp;N</oddFooter>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>